<commit_message>
fix the ranking issue
</commit_message>
<xml_diff>
--- a/exports/all_colleges.xlsx
+++ b/exports/all_colleges.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -433,11 +433,11 @@
     <col width="143" customWidth="1" min="7" max="7"/>
     <col width="253" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="169" customWidth="1" min="13" max="13"/>
-    <col width="157" customWidth="1" min="14" max="14"/>
+    <col width="80" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -558,7 +558,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>#3</t>
+          <t>CD Rank #3</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>#1</t>
+          <t>CD Rank #1</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>#2</t>
+          <t>CD Rank #2</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -719,78 +719,6 @@
       <c r="N4" t="inlineStr">
         <is>
           <t>Address: Vastrapur   India | Tel: 079-71523456 | Email: director@iima.ac.in</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>25621</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>National Law School of India University - [NLSIU], Bangalore</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>https://collegedunia.com/university/25621-national-law-school-of-india-university-nlsiu-bangalore</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>University</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Public</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>1986</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>the BCI. Ranking</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>CollegesQ</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>4.4</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>#4</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Naagarabhaavi</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Bangalore</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>NLSIU is a institute in Karnataka offering over 20 courses. Read for details on NLSIU Fees, Admission 2026, Courses, Placement, Ranking, Reviews and more</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Address: Gnana Bharathi Main Rd, Opp NAAC,
-Teachers Colony, Naagarabhaavi,
-Bengaluru, Karnataka   India | Tel: 080 23010000 | Email: contactus@nls.ac.in</t>
         </is>
       </c>
     </row>
@@ -805,15 +733,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L96"/>
+  <dimension ref="A1:L104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="75" customWidth="1" min="3" max="3"/>
+    <col width="75" customWidth="1" min="4" max="4"/>
     <col width="27" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="35" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
@@ -887,32 +815,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>25455</t>
+          <t>25446</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>M.Tech</t>
+          <t>M.Sc</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Computer Science And Engineering</t>
+          <t>Master of Science [M.Sc] (Clinical Embryology and Reproductive Biology)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Computer Science And Engineering</t>
+          <t>Master of Science [M.Sc] (Clinical Embryology and Reproductive Biology)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>5.06 Lakhs</t>
+          <t>2,830</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2 Years</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -927,7 +855,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>GATE</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -949,32 +877,32 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>25455</t>
+          <t>25446</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>M.Tech</t>
+          <t>B.Sc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Vlsi Design</t>
+          <t>Bachelor of Science [B.Sc] {Hons.} (Nursing)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Vlsi Design</t>
+          <t>Bachelor of Science [B.Sc] {Hons.} (Nursing)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>5.06 Lakhs</t>
+          <t>39,095</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2 Years</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -989,7 +917,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>GATE</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -1004,39 +932,39 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>UG</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>25455</t>
+          <t>25446</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>M.Tech</t>
+          <t>B.Sc</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Cyber Security</t>
+          <t>Bachelor of Science [B.Sc] (Medical Radiology \u0026 Imaging Technology)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Cyber Security</t>
+          <t>Bachelor of Science [B.Sc] (Medical Radiology \u0026 Imaging Technology)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>5.06 Lakhs</t>
+          <t>4,480</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2 Years</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1051,7 +979,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>GATE</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -1066,39 +994,39 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>UG</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>25455</t>
+          <t>25446</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>M.Tech</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Computer Technology</t>
+          <t>Doctor of Medicine [MD] (Medicine)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Computer Technology</t>
+          <t>Doctor of Medicine [MD] (Medicine)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>5.06 Lakhs</t>
+          <t>7,577</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2 Years</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1113,7 +1041,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>GATE</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -1128,7 +1056,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>UG</t>
         </is>
       </c>
     </row>
@@ -1145,12 +1073,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Construction Engineering And Management</t>
+          <t>Computer Science And Engineering</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Construction Engineering And Management</t>
+          <t>Computer Science And Engineering</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1207,12 +1135,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Biomedical Engineering</t>
+          <t>Vlsi Design</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Biomedical Engineering</t>
+          <t>Vlsi Design</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1269,12 +1197,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Environmental Engineering</t>
+          <t>Cyber Security</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Environmental Engineering</t>
+          <t>Cyber Security</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1331,12 +1259,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Mechanical Design</t>
+          <t>Computer Technology</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Mechanical Design</t>
+          <t>Computer Technology</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1393,12 +1321,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Textile Technology</t>
+          <t>Construction Engineering And Management</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Textile Technology</t>
+          <t>Construction Engineering And Management</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1455,12 +1383,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Power Electronics &amp; Machine Drives</t>
+          <t>Biomedical Engineering</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Power Electronics &amp; Machine Drives</t>
+          <t>Biomedical Engineering</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1517,12 +1445,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Integrated Circuit Technology</t>
+          <t>Environmental Engineering</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Integrated Circuit Technology</t>
+          <t>Environmental Engineering</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1579,12 +1507,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Instrumentation</t>
+          <t>Mechanical Design</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Instrumentation</t>
+          <t>Mechanical Design</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1641,12 +1569,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Material Science And Engineering</t>
+          <t>Textile Technology</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Material Science And Engineering</t>
+          <t>Textile Technology</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1703,12 +1631,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Chemical Engineering</t>
+          <t>Power Electronics &amp; Machine Drives</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Chemical Engineering</t>
+          <t>Power Electronics &amp; Machine Drives</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1765,12 +1693,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Electric Mobility</t>
+          <t>Integrated Circuit Technology</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Electric Mobility</t>
+          <t>Integrated Circuit Technology</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1827,12 +1755,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Structural Engineering</t>
+          <t>Instrumentation</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Structural Engineering</t>
+          <t>Instrumentation</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1889,12 +1817,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Polymer Science and Technology</t>
+          <t>Material Science And Engineering</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Polymer Science and Technology</t>
+          <t>Material Science And Engineering</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1951,12 +1879,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Optoelectronics And Optical Communication</t>
+          <t>Chemical Engineering</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Optoelectronics And Optical Communication</t>
+          <t>Chemical Engineering</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2013,12 +1941,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Water Resources Engineering</t>
+          <t>Electric Mobility</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Water Resources Engineering</t>
+          <t>Electric Mobility</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2075,12 +2003,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Control &amp; Automation</t>
+          <t>Structural Engineering</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Control &amp; Automation</t>
+          <t>Structural Engineering</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2137,12 +2065,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Renewable Energy Science and Technology</t>
+          <t>Polymer Science and Technology</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Renewable Energy Science and Technology</t>
+          <t>Polymer Science and Technology</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2199,12 +2127,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Engineering Analysis &amp; Design</t>
+          <t>Optoelectronics And Optical Communication</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Engineering Analysis &amp; Design</t>
+          <t>Optoelectronics And Optical Communication</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2261,12 +2189,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Radio Frequency Design and Technology</t>
+          <t>Water Resources Engineering</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Radio Frequency Design and Technology</t>
+          <t>Water Resources Engineering</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2323,12 +2251,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Biomolecular and Bioprocess Engineering</t>
+          <t>Control &amp; Automation</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Biomolecular and Bioprocess Engineering</t>
+          <t>Control &amp; Automation</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2385,12 +2313,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Rock Engineering And Underground Structures</t>
+          <t>Renewable Energy Science and Technology</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Rock Engineering And Underground Structures</t>
+          <t>Renewable Energy Science and Technology</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2447,12 +2375,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Solid State Materials</t>
+          <t>Engineering Analysis &amp; Design</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Solid State Materials</t>
+          <t>Engineering Analysis &amp; Design</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2509,12 +2437,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Transportation Engineering</t>
+          <t>Radio Frequency Design and Technology</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Transportation Engineering</t>
+          <t>Radio Frequency Design and Technology</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2571,12 +2499,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Applied Optics</t>
+          <t>Biomolecular and Bioprocess Engineering</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Applied Optics</t>
+          <t>Biomolecular and Bioprocess Engineering</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2633,12 +2561,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Thermal Engineering</t>
+          <t>Rock Engineering And Underground Structures</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Thermal Engineering</t>
+          <t>Rock Engineering And Underground Structures</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2695,12 +2623,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Production Engineering</t>
+          <t>Solid State Materials</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Production Engineering</t>
+          <t>Solid State Materials</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2757,12 +2685,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Atmospheric-Oceanic Science and Technology</t>
+          <t>Transportation Engineering</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Atmospheric-Oceanic Science and Technology</t>
+          <t>Transportation Engineering</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2819,12 +2747,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Power System Engineering</t>
+          <t>Applied Optics</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Power System Engineering</t>
+          <t>Applied Optics</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2881,12 +2809,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Energy Studies</t>
+          <t>Thermal Engineering</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Energy Studies</t>
+          <t>Thermal Engineering</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2943,12 +2871,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Electronics Circuit &amp; System</t>
+          <t>Production Engineering</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Electronics Circuit &amp; System</t>
+          <t>Production Engineering</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3005,12 +2933,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Telecommunication Engineering</t>
+          <t>Atmospheric-Oceanic Science and Technology</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Telecommunication Engineering</t>
+          <t>Atmospheric-Oceanic Science and Technology</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3067,12 +2995,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Applied Mechanics</t>
+          <t>Power System Engineering</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Applied Mechanics</t>
+          <t>Power System Engineering</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3129,12 +3057,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Fibre Science and Technology</t>
+          <t>Energy Studies</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Fibre Science and Technology</t>
+          <t>Energy Studies</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3191,12 +3119,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Construction Technology</t>
+          <t>Electronics Circuit &amp; System</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Construction Technology</t>
+          <t>Electronics Circuit &amp; System</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3253,12 +3181,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Industrial Engineering</t>
+          <t>Telecommunication Engineering</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Industrial Engineering</t>
+          <t>Telecommunication Engineering</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3315,12 +3243,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Communication Systems</t>
+          <t>Applied Mechanics</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Communication Systems</t>
+          <t>Applied Mechanics</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3377,12 +3305,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Computing and Intelligent Systems Engineering</t>
+          <t>Fibre Science and Technology</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Computing and Intelligent Systems Engineering</t>
+          <t>Fibre Science and Technology</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3439,12 +3367,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Energy Science and Engineering</t>
+          <t>Construction Technology</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Energy Science and Engineering</t>
+          <t>Construction Technology</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -3501,12 +3429,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Geotechnical And Geoenvirnomental Engineering</t>
+          <t>Industrial Engineering</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Geotechnical And Geoenvirnomental Engineering</t>
+          <t>Industrial Engineering</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -3563,12 +3491,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Molecular Engineering &amp; Advanced Chemical Analysis</t>
+          <t>Communication Systems</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Molecular Engineering &amp; Advanced Chemical Analysis</t>
+          <t>Communication Systems</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -3625,12 +3553,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Photonics</t>
+          <t>Computing and Intelligent Systems Engineering</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Photonics</t>
+          <t>Computing and Intelligent Systems Engineering</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -3687,12 +3615,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Smart and Sustainable Power Systems</t>
+          <t>Energy Science and Engineering</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Smart and Sustainable Power Systems</t>
+          <t>Energy Science and Engineering</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -3749,12 +3677,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Systems, Learning &amp; Control</t>
+          <t>Geotechnical And Geoenvirnomental Engineering</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Systems, Learning &amp; Control</t>
+          <t>Geotechnical And Geoenvirnomental Engineering</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -3806,27 +3734,27 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>B.Tech</t>
+          <t>M.Tech</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Computer Science and Engineering</t>
+          <t>Molecular Engineering &amp; Advanced Chemical Analysis</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Computer Science and Engineering</t>
+          <t>Molecular Engineering &amp; Advanced Chemical Analysis</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>11.74 Lakhs</t>
+          <t>5.06 Lakhs</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>4 Years</t>
+          <t>2 Years</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3841,7 +3769,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>JEE Advanced</t>
+          <t>GATE</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -3856,7 +3784,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -3868,27 +3796,27 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>B.Tech</t>
+          <t>M.Tech</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Mathematics And Computing</t>
+          <t>Photonics</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Mathematics And Computing</t>
+          <t>Photonics</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>11.74 Lakhs</t>
+          <t>5.06 Lakhs</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>4 Years</t>
+          <t>2 Years</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3903,7 +3831,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>JEE Advanced</t>
+          <t>GATE</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -3918,7 +3846,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -3930,27 +3858,27 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>B.Tech</t>
+          <t>M.Tech</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Engineering and Computational Mechanics</t>
+          <t>Smart and Sustainable Power Systems</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Engineering and Computational Mechanics</t>
+          <t>Smart and Sustainable Power Systems</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>11.74 Lakhs</t>
+          <t>5.06 Lakhs</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>4 Years</t>
+          <t>2 Years</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3965,7 +3893,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>JEE Advanced</t>
+          <t>GATE</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -3980,7 +3908,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -3992,27 +3920,27 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>B.Tech</t>
+          <t>M.Tech</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Electrical Engineering [Power And Automation]</t>
+          <t>Systems, Learning &amp; Control</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Electrical Engineering [Power And Automation]</t>
+          <t>Systems, Learning &amp; Control</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>11.74 Lakhs</t>
+          <t>5.06 Lakhs</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>4 Years</t>
+          <t>2 Years</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -4027,7 +3955,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>JEE Advanced</t>
+          <t>GATE</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -4042,7 +3970,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -4059,12 +3987,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Biotechnology And Biochemical Engineering</t>
+          <t>Computer Science and Engineering</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Biotechnology And Biochemical Engineering</t>
+          <t>Computer Science and Engineering</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -4121,12 +4049,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Mechanical Engineering</t>
+          <t>Mathematics And Computing</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Mechanical Engineering</t>
+          <t>Mathematics And Computing</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -4183,12 +4111,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Chemical Engineering</t>
+          <t>Engineering and Computational Mechanics</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Chemical Engineering</t>
+          <t>Engineering and Computational Mechanics</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -4245,12 +4173,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Engineering Physics</t>
+          <t>Electrical Engineering [Power And Automation]</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Engineering Physics</t>
+          <t>Electrical Engineering [Power And Automation]</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -4307,12 +4235,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Industrial &amp; Production Engineering</t>
+          <t>Biotechnology And Biochemical Engineering</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Industrial &amp; Production Engineering</t>
+          <t>Biotechnology And Biochemical Engineering</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -4369,12 +4297,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Mechanical Engineering</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Mechanical Engineering</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -4431,12 +4359,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Chemical Engineering</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Chemical Engineering</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -4493,12 +4421,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Design Engineering</t>
+          <t>Engineering Physics</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Design Engineering</t>
+          <t>Engineering Physics</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -4555,12 +4483,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Energy Engineering</t>
+          <t>Industrial &amp; Production Engineering</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Energy Engineering</t>
+          <t>Industrial &amp; Production Engineering</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -4617,12 +4545,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Material Science Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Material Science Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -4679,12 +4607,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Power and Automation</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Power and Automation</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -4736,27 +4664,27 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>M.Sc</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Machine Intelligence &amp; Data Science</t>
+          <t>Design Engineering</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Machine Intelligence &amp; Data Science</t>
+          <t>Design Engineering</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>5.07 Lakhs</t>
+          <t>11.74 Lakhs</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>2 Years</t>
+          <t>4 Years</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -4771,7 +4699,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>IIT JAM</t>
+          <t>JEE Advanced</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -4786,7 +4714,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>UG</t>
         </is>
       </c>
     </row>
@@ -4798,27 +4726,27 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>M.Sc</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Biochemical Engineering and Biotechnology</t>
+          <t>Energy Engineering</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Biochemical Engineering and Biotechnology</t>
+          <t>Energy Engineering</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>5.07 Lakhs</t>
+          <t>11.74 Lakhs</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2 Years</t>
+          <t>4 Years</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -4833,7 +4761,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>IIT JAM</t>
+          <t>JEE Advanced</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -4848,7 +4776,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>UG</t>
         </is>
       </c>
     </row>
@@ -4860,27 +4788,27 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>M.Sc</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Computer Science and Engineering</t>
+          <t>Material Science Engineering</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Computer Science and Engineering</t>
+          <t>Material Science Engineering</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>5.07 Lakhs</t>
+          <t>11.74 Lakhs</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>2 Years</t>
+          <t>4 Years</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -4895,7 +4823,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>IIT JAM</t>
+          <t>JEE Advanced</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -4910,7 +4838,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>UG</t>
         </is>
       </c>
     </row>
@@ -4922,27 +4850,27 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>M.Sc</t>
+          <t>B.Tech</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Biological Science</t>
+          <t>Power and Automation</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Biological Science</t>
+          <t>Power and Automation</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>5.07 Lakhs</t>
+          <t>11.74 Lakhs</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2 Years</t>
+          <t>4 Years</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -4957,7 +4885,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>IIT JAM</t>
+          <t>JEE Advanced</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -4972,7 +4900,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>UG</t>
         </is>
       </c>
     </row>
@@ -4989,12 +4917,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Machine Intelligence &amp; Data Science</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Civil Engineering</t>
+          <t>Machine Intelligence &amp; Data Science</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -5051,12 +4979,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Biochemical Engineering and Biotechnology</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Biochemical Engineering and Biotechnology</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -5113,12 +5041,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Computer Science and Engineering</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Computer Science and Engineering</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -5175,12 +5103,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Telecommunication Technology And Management</t>
+          <t>Biological Science</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Telecommunication Technology And Management</t>
+          <t>Biological Science</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -5237,12 +5165,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Sensors, Instrumentation and Cyber-Physical Systems Engineering</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Sensors, Instrumentation and Cyber-Physical Systems Engineering</t>
+          <t>Civil Engineering</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -5299,12 +5227,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Transportation Safety and Injury Prevention</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Transportation Safety and Injury Prevention</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -5361,12 +5289,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Applied Mechanics</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Applied Mechanics</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -5423,12 +5351,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Automotive Research and Tribology</t>
+          <t>Telecommunication Technology And Management</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Automotive Research and Tribology</t>
+          <t>Telecommunication Technology And Management</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -5485,12 +5413,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Chemical Engineering</t>
+          <t>Sensors, Instrumentation and Cyber-Physical Systems Engineering</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Chemical Engineering</t>
+          <t>Sensors, Instrumentation and Cyber-Physical Systems Engineering</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -5547,12 +5475,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Transportation Safety and Injury Prevention</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Transportation Safety and Injury Prevention</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -5609,12 +5537,12 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Materials Science and Engineering</t>
+          <t>Applied Mechanics</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Materials Science and Engineering</t>
+          <t>Applied Mechanics</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -5671,12 +5599,12 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Photonics Science and Engineering</t>
+          <t>Automotive Research and Tribology</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Photonics Science and Engineering</t>
+          <t>Automotive Research and Tribology</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -5733,12 +5661,12 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>VLSI Design Tools &amp; Technology</t>
+          <t>Chemical Engineering</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>VLSI Design Tools &amp; Technology</t>
+          <t>Chemical Engineering</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -5790,27 +5718,27 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Ph.D</t>
+          <t>M.Sc</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Ph.D (General)</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>1.58 Lakhs - 5.07 Lakhs</t>
+          <t>5.07 Lakhs</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>3-5 Years</t>
+          <t>2 Years</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -5825,7 +5753,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>GATE / UGC NET</t>
+          <t>IIT JAM</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -5840,7 +5768,7 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>Doctorate</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -5852,27 +5780,27 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Ph.D</t>
+          <t>M.Sc</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Artificial Intelligence</t>
+          <t>Materials Science and Engineering</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Artificial Intelligence</t>
+          <t>Materials Science and Engineering</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>3.4 Lakhs</t>
+          <t>5.07 Lakhs</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>3-5 Years</t>
+          <t>2 Years</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -5882,12 +5810,12 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Postgraduation in relevant field</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>GATE / UGC NET</t>
+          <t>IIT JAM</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -5902,7 +5830,7 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>Doctorate</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -5914,27 +5842,27 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Ph.D</t>
+          <t>M.Sc</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Photonics Science and Engineering</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Photonics Science and Engineering</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>3.4 Lakhs</t>
+          <t>5.07 Lakhs</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>3-5 Years</t>
+          <t>2 Years</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -5944,12 +5872,12 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Postgraduation in relevant field</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>GATE / UGC NET</t>
+          <t>IIT JAM</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -5964,7 +5892,7 @@
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>Doctorate</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -5976,27 +5904,27 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Ph.D</t>
+          <t>M.Sc</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Humanities And Social Science</t>
+          <t>VLSI Design Tools &amp; Technology</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Humanities And Social Science</t>
+          <t>VLSI Design Tools &amp; Technology</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>3.4 Lakhs</t>
+          <t>5.07 Lakhs</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>3-5 Years</t>
+          <t>2 Years</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -6006,12 +5934,12 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Postgraduation in relevant field</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>GATE / UGC NET</t>
+          <t>IIT JAM</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -6026,7 +5954,7 @@
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>Doctorate</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -6043,17 +5971,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Public Policy</t>
+          <t>Ph.D (General)</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Public Policy</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>3.4 Lakhs</t>
+          <t>1.58 Lakhs - 5.07 Lakhs</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -6068,7 +5996,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Postgraduation in relevant field</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -6100,27 +6028,27 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>MPP</t>
+          <t>Ph.D</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>MPP (General)</t>
+          <t>Artificial Intelligence</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Artificial Intelligence</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>2.36 Lakhs - 5.06 Lakhs</t>
+          <t>3.4 Lakhs</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>2 Years</t>
+          <t>3-5 Years</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -6130,12 +6058,12 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>Postgraduation in relevant field</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>GATE / UGC NET</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -6150,7 +6078,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>Doctorate</t>
         </is>
       </c>
     </row>
@@ -6162,27 +6090,27 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>MBA</t>
+          <t>Ph.D</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>MBA (General)</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>12.4 Lakhs - 14.06 Lakhs</t>
+          <t>3.4 Lakhs</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>2 Years</t>
+          <t>3-5 Years</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -6192,12 +6120,12 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>Postgraduation in relevant field</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>GATE / UGC NET</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -6212,7 +6140,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>Doctorate</t>
         </is>
       </c>
     </row>
@@ -6224,27 +6152,27 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>MBA</t>
+          <t>Ph.D</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Humanities And Social Science</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Humanities And Social Science</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>12.4 Lakhs - 14.06 Lakhs</t>
+          <t>3.4 Lakhs</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>2 Years</t>
+          <t>3-5 Years</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -6254,12 +6182,12 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Graduation with 60%+</t>
+          <t>Postgraduation in relevant field</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>GATE / UGC NET</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -6274,7 +6202,7 @@
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>Doctorate</t>
         </is>
       </c>
     </row>
@@ -6286,27 +6214,27 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>MBA</t>
+          <t>Ph.D</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Telecommunication Systems Management</t>
+          <t>Public Policy</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Telecommunication Systems Management</t>
+          <t>Public Policy</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>12.4 Lakhs - 14.06 Lakhs</t>
+          <t>3.4 Lakhs</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>2 Years</t>
+          <t>3-5 Years</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -6316,12 +6244,12 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Graduation with 60%+</t>
+          <t>Postgraduation in relevant field</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>GATE / UGC NET</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -6336,7 +6264,7 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>Doctorate</t>
         </is>
       </c>
     </row>
@@ -6348,12 +6276,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>B.Des</t>
+          <t>MPP</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>B.Des (General)</t>
+          <t>MPP (General)</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -6363,12 +6291,12 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>11.74 Lakhs</t>
+          <t>2.36 Lakhs - 5.06 Lakhs</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>4 Years</t>
+          <t>2 Years</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -6383,7 +6311,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>UCEED</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -6398,7 +6326,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -6410,12 +6338,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>M.Des</t>
+          <t>MBA</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>M.Des (General)</t>
+          <t>MBA (General)</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -6425,7 +6353,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>2.76 Lakhs</t>
+          <t>12.4 Lakhs - 14.06 Lakhs</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -6445,7 +6373,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>CEED</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -6472,12 +6400,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Executive Programme</t>
+          <t>MBA</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Executive Programme (General)</t>
+          <t>General</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -6487,27 +6415,27 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>1.2 Lakhs - 1.79 Lakhs</t>
+          <t>12.4 Lakhs - 14.06 Lakhs</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>1 Year</t>
+          <t>2 Years</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Part Time</t>
+          <t>Full Time</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>Graduation with 60%+</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -6534,22 +6462,22 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>EMBA</t>
+          <t>MBA</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>EMBA (General)</t>
+          <t>Telecommunication Systems Management</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Telecommunication Systems Management</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>16.32 Lakhs - 18 Lakhs</t>
+          <t>12.4 Lakhs - 14.06 Lakhs</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -6559,12 +6487,12 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Part Time</t>
+          <t>Full Time</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>Graduation with 60%+</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6596,32 +6524,32 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Executive Programme (CEP)</t>
+          <t>B.Des</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Executive Management Program in Strategic Management</t>
+          <t>B.Des (General)</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Executive Management Program in Strategic Management</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>11.74 Lakhs</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>1 Year</t>
+          <t>4 Years</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Part Time</t>
+          <t>Full Time</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -6631,7 +6559,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>UCEED</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -6646,7 +6574,7 @@
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>UG</t>
         </is>
       </c>
     </row>
@@ -6658,32 +6586,32 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Executive Programme (CEP)</t>
+          <t>M.Des</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Executive Management Program in Human Resource Strategic Management</t>
+          <t>M.Des (General)</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Executive Management Program in Human Resource Strategic Management</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>2.76 Lakhs</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>1 Year</t>
+          <t>2 Years</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Part Time</t>
+          <t>Full Time</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -6693,7 +6621,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>CEED</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -6720,55 +6648,551 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
+          <t>Executive Programme</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Executive Programme (General)</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>1.2 Lakhs - 1.79 Lakhs</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>1 Year</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Part Time</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>25455</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>EMBA</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>EMBA (General)</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>16.32 Lakhs - 18 Lakhs</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Part Time</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>CAT</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>25455</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
           <t>Executive Programme (CEP)</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Executive Management Program in Strategic Management</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Executive Management Program in Strategic Management</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>1 Year</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Part Time</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>25455</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Executive Programme (CEP)</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Executive Management Program in Human Resource Strategic Management</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Executive Management Program in Human Resource Strategic Management</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>1 Year</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Part Time</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>25455</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Executive Programme (CEP)</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
         <is>
           <t>Executive Program in Robotics</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr">
+      <c r="D100" t="inlineStr">
         <is>
           <t>Executive Program in Robotics</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>Not Specified</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr">
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
         <is>
           <t>1 Year</t>
         </is>
       </c>
-      <c r="G96" t="inlineStr">
+      <c r="G100" t="inlineStr">
         <is>
           <t>Part Time</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr">
-        <is>
-          <t>Not Specified</t>
-        </is>
-      </c>
-      <c r="I96" t="inlineStr">
-        <is>
-          <t>Not Specified</t>
-        </is>
-      </c>
-      <c r="J96" t="inlineStr">
-        <is>
-          <t>Not Specified</t>
-        </is>
-      </c>
-      <c r="K96" t="inlineStr">
-        <is>
-          <t>Not Specified</t>
-        </is>
-      </c>
-      <c r="L96" t="inlineStr">
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>25494</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>MBA</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Post Graduate Programme in Food and Agri-Business Management [PGP-FABM]</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Post Graduate Programme in Food and Agri-Business Management [PGP-FABM]</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>27.5 Lakhs</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>25494</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>MBA</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Master of Business Administration [MBA]</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Master of Business Administration [MBA]</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>20 Lakhs</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>25494</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Ph.D</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Ph.D. (Management)</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Ph.D. (Management)</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>25494</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>MBA</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Post Graduate Programme in Management [PGPM]</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Post Graduate Programme in Management [PGPM]</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>27.5 Lakhs</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
         <is>
           <t>PG</t>
         </is>
@@ -6785,12 +7209,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="287" customWidth="1" min="2" max="2"/>
-    <col width="299" customWidth="1" min="3" max="3"/>
+    <col width="172" customWidth="1" min="3" max="3"/>
     <col width="266" customWidth="1" min="4" max="4"/>
     <col width="372" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
@@ -6919,38 +7343,6 @@
         </is>
       </c>
       <c r="F4" t="inlineStr">
-        <is>
-          <t>Not Specified</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>25621</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>National Law School of India University (NLSIU), Bangalore admits students through CLAT, CLAT-PG, or NLSAT, depending on the programme. Admissions are merit-based, subject to eligibility, reservations, and seat availability, and finalized through the prescribed counselling process.</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Since NLSIU Bangalore is currently the top NLU in India, with an NIRF rank of #1, you will have to put in a lot of work. There will be 120 questions in the exam overall. The questions will be based on the updated CLAT Exam Pattern. Here's how you can prepare for CLAT to get into NLSIU Bangalore:</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Not Specified</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Yes, NLSIU accepts a valid score in CLAT PG for admission to its one-year LLM degree program. For admission into the postgraduate LLM programme, the candidate must take the Common Law Admission Test (CLAT-PG), and achieve the required cutoff for the respective academic year.</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
         <is>
           <t>Not Specified</t>
         </is>
@@ -6967,7 +7359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -7082,17 +7474,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1.32 Cr</t>
+          <t>1.15 CPA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>27.60 LPA</t>
+          <t>35.07 LPA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>36.2 LPA</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -7102,39 +7494,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>25621</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>18 LPA</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>16 LPA</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>16.50 LPA</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>100% placement</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Not Specified</t>
+          <t>Microsoft, Google, Accenture, TCS, Wipro, HCL, Goldman Sachs, Flipkart</t>
         </is>
       </c>
     </row>
@@ -7149,12 +7509,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -7193,7 +7553,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>#1</t>
+          <t>CD Rank #3</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -7211,12 +7571,10 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>#1</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>2025</v>
-      </c>
+          <t>CD Rank #1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7231,30 +7589,10 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>#1</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>2025</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>25621</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Collegedunia</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>#4</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
+          <t>CD Rank #2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7351,7 +7689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -7424,23 +7762,6 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>Gym, Laundry, Mess, Single Occupancy, Sports</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>25621</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026, </t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Laundry, Mess</t>
         </is>
       </c>
     </row>
@@ -7455,7 +7776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -7546,26 +7867,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>25621</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Aditya Sharma</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Excellent academic atmosphere, world class research facilities, and amazing placements.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>